<commit_message>
upload the notebook with a preliminary run with energy
</commit_message>
<xml_diff>
--- a/ssp_modeling/transformations/templates/calibrated/uganda/model_input_variables_uganda_ce_calibrated.xlsx
+++ b/ssp_modeling/transformations/templates/calibrated/uganda/model_input_variables_uganda_ce_calibrated.xlsx
@@ -20679,7 +20679,7 @@
         <v>173</v>
       </c>
       <c r="C107">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="H107">
         <v>1</v>
@@ -20864,7 +20864,7 @@
         <v>174</v>
       </c>
       <c r="C108">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="H108">
         <v>1</v>
@@ -21049,7 +21049,7 @@
         <v>175</v>
       </c>
       <c r="C109">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="H109">
         <v>1</v>
@@ -21234,7 +21234,7 @@
         <v>176</v>
       </c>
       <c r="C110">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="H110">
         <v>1</v>
@@ -21419,7 +21419,7 @@
         <v>177</v>
       </c>
       <c r="C111">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="H111">
         <v>1</v>
@@ -21604,7 +21604,7 @@
         <v>178</v>
       </c>
       <c r="C112">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="H112">
         <v>1</v>
@@ -21789,7 +21789,7 @@
         <v>179</v>
       </c>
       <c r="C113">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="H113">
         <v>1</v>
@@ -21974,7 +21974,7 @@
         <v>180</v>
       </c>
       <c r="C114">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="H114">
         <v>1</v>
@@ -22159,7 +22159,7 @@
         <v>181</v>
       </c>
       <c r="C115">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="H115">
         <v>1</v>
@@ -22344,7 +22344,7 @@
         <v>182</v>
       </c>
       <c r="C116">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="H116">
         <v>1</v>
@@ -22529,7 +22529,7 @@
         <v>183</v>
       </c>
       <c r="C117">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="H117">
         <v>1</v>
@@ -22714,7 +22714,7 @@
         <v>184</v>
       </c>
       <c r="C118">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="H118">
         <v>1</v>
@@ -22899,7 +22899,7 @@
         <v>185</v>
       </c>
       <c r="C119">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="H119">
         <v>1</v>
@@ -23084,7 +23084,7 @@
         <v>186</v>
       </c>
       <c r="C120">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H120">
         <v>1</v>
@@ -23269,7 +23269,7 @@
         <v>187</v>
       </c>
       <c r="C121">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H121">
         <v>1</v>
@@ -23454,7 +23454,7 @@
         <v>188</v>
       </c>
       <c r="C122">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H122">
         <v>1</v>
@@ -23639,7 +23639,7 @@
         <v>189</v>
       </c>
       <c r="C123">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H123">
         <v>1</v>
@@ -23824,7 +23824,7 @@
         <v>190</v>
       </c>
       <c r="C124">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H124">
         <v>1</v>
@@ -24009,7 +24009,7 @@
         <v>191</v>
       </c>
       <c r="C125">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H125">
         <v>1</v>
@@ -24194,7 +24194,7 @@
         <v>192</v>
       </c>
       <c r="C126">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H126">
         <v>1</v>
@@ -24379,7 +24379,7 @@
         <v>193</v>
       </c>
       <c r="C127">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H127">
         <v>1</v>
@@ -24564,7 +24564,7 @@
         <v>194</v>
       </c>
       <c r="C128">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H128">
         <v>1</v>
@@ -24749,7 +24749,7 @@
         <v>195</v>
       </c>
       <c r="C129">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H129">
         <v>1</v>
@@ -24934,7 +24934,7 @@
         <v>196</v>
       </c>
       <c r="C130">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H130">
         <v>1</v>
@@ -25119,7 +25119,7 @@
         <v>197</v>
       </c>
       <c r="C131">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H131">
         <v>1</v>
@@ -25304,7 +25304,7 @@
         <v>198</v>
       </c>
       <c r="C132">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H132">
         <v>1</v>

</xml_diff>

<commit_message>
preliminary run with new data finished
</commit_message>
<xml_diff>
--- a/ssp_modeling/transformations/templates/calibrated/uganda/model_input_variables_uganda_ce_calibrated.xlsx
+++ b/ssp_modeling/transformations/templates/calibrated/uganda/model_input_variables_uganda_ce_calibrated.xlsx
@@ -20681,7 +20681,7 @@
         <v>173</v>
       </c>
       <c r="C107">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H107">
         <v>1</v>
@@ -20866,7 +20866,7 @@
         <v>174</v>
       </c>
       <c r="C108">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H108">
         <v>1</v>
@@ -21051,7 +21051,7 @@
         <v>175</v>
       </c>
       <c r="C109">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H109">
         <v>1</v>
@@ -21236,7 +21236,7 @@
         <v>176</v>
       </c>
       <c r="C110">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H110">
         <v>1</v>
@@ -21421,7 +21421,7 @@
         <v>177</v>
       </c>
       <c r="C111">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H111">
         <v>1</v>
@@ -21606,7 +21606,7 @@
         <v>178</v>
       </c>
       <c r="C112">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H112">
         <v>1</v>
@@ -21791,7 +21791,7 @@
         <v>179</v>
       </c>
       <c r="C113">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H113">
         <v>1</v>
@@ -21976,7 +21976,7 @@
         <v>180</v>
       </c>
       <c r="C114">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H114">
         <v>1</v>
@@ -22161,7 +22161,7 @@
         <v>181</v>
       </c>
       <c r="C115">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H115">
         <v>1</v>
@@ -22346,7 +22346,7 @@
         <v>182</v>
       </c>
       <c r="C116">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H116">
         <v>1</v>
@@ -22531,7 +22531,7 @@
         <v>183</v>
       </c>
       <c r="C117">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H117">
         <v>1</v>
@@ -22716,7 +22716,7 @@
         <v>184</v>
       </c>
       <c r="C118">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H118">
         <v>1</v>
@@ -22901,7 +22901,7 @@
         <v>185</v>
       </c>
       <c r="C119">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H119">
         <v>1</v>
@@ -23086,7 +23086,7 @@
         <v>186</v>
       </c>
       <c r="C120">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H120">
         <v>1</v>
@@ -23271,7 +23271,7 @@
         <v>187</v>
       </c>
       <c r="C121">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H121">
         <v>1</v>
@@ -23456,7 +23456,7 @@
         <v>188</v>
       </c>
       <c r="C122">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H122">
         <v>1</v>
@@ -23641,7 +23641,7 @@
         <v>189</v>
       </c>
       <c r="C123">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H123">
         <v>1</v>
@@ -23826,7 +23826,7 @@
         <v>190</v>
       </c>
       <c r="C124">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H124">
         <v>1</v>
@@ -24011,7 +24011,7 @@
         <v>191</v>
       </c>
       <c r="C125">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H125">
         <v>1</v>
@@ -24196,7 +24196,7 @@
         <v>192</v>
       </c>
       <c r="C126">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H126">
         <v>1</v>
@@ -24381,7 +24381,7 @@
         <v>193</v>
       </c>
       <c r="C127">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H127">
         <v>1</v>
@@ -24566,7 +24566,7 @@
         <v>194</v>
       </c>
       <c r="C128">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H128">
         <v>1</v>
@@ -24751,7 +24751,7 @@
         <v>195</v>
       </c>
       <c r="C129">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H129">
         <v>1</v>
@@ -24936,7 +24936,7 @@
         <v>196</v>
       </c>
       <c r="C130">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H130">
         <v>1</v>
@@ -25121,7 +25121,7 @@
         <v>197</v>
       </c>
       <c r="C131">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H131">
         <v>1</v>
@@ -25306,7 +25306,7 @@
         <v>198</v>
       </c>
       <c r="C132">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H132">
         <v>1</v>

</xml_diff>